<commit_message>
fix: PI模板多项修改 (2026-03-07 01:50)
1. 第4行Contact电话改为177-2781-0735
2. PAYMENT METHOD字体大小改为8.5
3. 银行信息顺序调整并更新内容:
   - Account Number: 06201739597884
   - Account Name: Hong Kong Unicorn Technology Limited
   - Bank Code: 003
   - Bank Name: IBK - Industrial Bank of Korea
   - Bank Address: 91, Ogeum-ro, Songpa-gu, Seoul, Korea Industrial Bank of Korea Jamsil Branch
   - Country/Region: Korea (新增)
   - Type of Account: Business account
4. 删除Bank charges警告行
5. THANK YOU行整行合并

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/openclaw_skills/order-pi-generator/template/Proforma_Invoice_TAEJU_UNI2025110502_v2.xlsx
+++ b/openclaw_skills/order-pi-generator/template/Proforma_Invoice_TAEJU_UNI2025110502_v2.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="36">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -263,8 +263,19 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -491,6 +502,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2A4A"/>
+        <bgColor rgb="001B2A4A"/>
       </patternFill>
     </fill>
   </fills>
@@ -852,7 +869,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -941,6 +958,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1429,7 +1456,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Contact: Joy Kim   |   joy@unicornsemi.com   |   (+86) 189-2372-9010</t>
+          <t>Contact: Joy Kim   |   joy@unicornsemi.com   |   (+86) 177-2781-0735</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1748,7 @@
     </row>
     <row r="29" ht="12" customHeight="1"/>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t>PAYMENT METHOD – BANK TRANSFER</t>
         </is>
@@ -1730,48 +1757,48 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>Account Name:</t>
+          <t>Account Number:</t>
         </is>
       </c>
       <c r="D31" s="28" t="inlineStr">
         <is>
-          <t>Hong Kong Unicorn Technology Limited</t>
+          <t>06201739597884</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>Account Number:</t>
+          <t>Account Name:</t>
         </is>
       </c>
       <c r="D32" s="28" t="inlineStr">
         <is>
-          <t>06201739597884</t>
+          <t>Hong Kong Unicorn Technology Limited</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>Bank Name:</t>
+          <t>Bank Code:</t>
         </is>
       </c>
       <c r="D33" s="28" t="inlineStr">
         <is>
-          <t>IBK – Industrial Bank of Korea</t>
+          <t>003</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>Bank Code:</t>
+          <t>Bank Name:</t>
         </is>
       </c>
       <c r="D34" s="28" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>IBK - Industrial Bank of Korea</t>
         </is>
       </c>
     </row>
@@ -1783,32 +1810,37 @@
       </c>
       <c r="D35" s="28" t="inlineStr">
         <is>
-          <t>91, Ogeum-ro, Songpa-gu, Seoul, Korea (Jamsil Branch)</t>
+          <t>91, Ogeum-ro, Songpa-gu, Seoul, Korea Industrial Bank of Korea Jamsil Branch</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="27" t="inlineStr">
-        <is>
-          <t>Account Type:</t>
-        </is>
-      </c>
-      <c r="D36" s="28" t="inlineStr">
-        <is>
-          <t>Business Account</t>
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Country/Region:</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>Korea</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="29" t="inlineStr">
-        <is>
-          <t>⚠  Bank charges are to be borne by the remitter.</t>
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>Type of Account:</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Business account</t>
         </is>
       </c>
     </row>
     <row r="38" ht="12" customHeight="1"/>
     <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="30" t="inlineStr">
+      <c r="A39" s="35" t="inlineStr">
         <is>
           <t>THANK YOU FOR YOUR BUSINESS!</t>
         </is>
@@ -1830,13 +1862,14 @@
     <row r="53" ht="16" customHeight="1"/>
     <row r="54" ht="16" customHeight="1"/>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="D35:H35"/>
     <mergeCell ref="C16:H16"/>
-    <mergeCell ref="A39:H39"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="D34:H34"/>
+    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="D31:H31"/>
@@ -1854,7 +1887,6 @@
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A26:H26"/>
@@ -1862,6 +1894,7 @@
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D37:H37"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A1:H2"/>

</xml_diff>